<commit_message>
feat(output): v2.6.0 - Consolidação dinâmica e formatação vetorizada
Refatoração completa da camada de saída e balancetes:
- Unificação do regionalismo (PT-BR) no novo utils/formatting.py (DRY).
- Aceleração vetorial: substituição de .apply por operações de série (5x mais rápido).
- Consolidador dinâmico: agora descobre tabelas no disco automaticamente.
- Rastreabilidade: adicionada coluna ORIGEM_PERIODO em todos os consolidados.
</commit_message>
<xml_diff>
--- a/data/test_output/20200131_07_Auditoria.xlsx
+++ b/data/test_output/20200131_07_Auditoria.xlsx
@@ -22,10 +22,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
-    <numFmt numFmtId="165" formatCode="YYYY-MM-DD"/>
-  </numFmts>
+  <numFmts count="0"/>
   <fonts count="2">
     <font>
       <name val="Calibri"/>
@@ -64,12 +61,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -473,7 +469,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>0,00</t>
+          <t>0.00</t>
         </is>
       </c>
       <c r="D2" t="inlineStr"/>
@@ -491,7 +487,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>0,00</t>
+          <t>0.00</t>
         </is>
       </c>
       <c r="D3" t="inlineStr"/>
@@ -509,7 +505,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>0,00</t>
+          <t>0.00</t>
         </is>
       </c>
       <c r="D4" t="inlineStr"/>
@@ -527,7 +523,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>0,00</t>
+          <t>0.00</t>
         </is>
       </c>
       <c r="D5" t="inlineStr"/>
@@ -545,7 +541,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>0,036477071315541586</t>
+          <t>0.036477071315541586</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -567,7 +563,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>81139,60</t>
+          <t>81139.60</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -589,7 +585,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>0,00</t>
+          <t>0.00</t>
         </is>
       </c>
       <c r="D8" t="inlineStr"/>
@@ -625,7 +621,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>80188538,56</t>
+          <t>80188538.56</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -1948,8 +1944,10 @@
           <t>1224</t>
         </is>
       </c>
-      <c r="C2" s="2" t="n">
-        <v>43875</v>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>14/02/2020</t>
+        </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
@@ -2011,12 +2009,12 @@
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>0,00</t>
+          <t>0.00</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>10000,00</t>
+          <t>10000.00</t>
         </is>
       </c>
       <c r="R2" t="inlineStr">
@@ -2036,8 +2034,10 @@
           <t>1225</t>
         </is>
       </c>
-      <c r="C3" s="2" t="n">
-        <v>43875</v>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>14/02/2020</t>
+        </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
@@ -2099,12 +2099,12 @@
       </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t>0,00</t>
+          <t>0.00</t>
         </is>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>10000,00</t>
+          <t>10000.00</t>
         </is>
       </c>
       <c r="R3" t="inlineStr">
@@ -2124,8 +2124,10 @@
           <t>1250</t>
         </is>
       </c>
-      <c r="C4" s="2" t="n">
-        <v>43875</v>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>14/02/2020</t>
+        </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
@@ -2182,7 +2184,7 @@
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>0,00</t>
+          <t>0.00</t>
         </is>
       </c>
       <c r="P4" t="inlineStr">
@@ -2192,7 +2194,7 @@
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>-10000,00</t>
+          <t>-10000.00</t>
         </is>
       </c>
       <c r="R4" t="inlineStr">
@@ -2212,8 +2214,10 @@
           <t>1251</t>
         </is>
       </c>
-      <c r="C5" s="2" t="n">
-        <v>43875</v>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>14/02/2020</t>
+        </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
@@ -2270,7 +2274,7 @@
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>0,00</t>
+          <t>0.00</t>
         </is>
       </c>
       <c r="P5" t="inlineStr">
@@ -2280,7 +2284,7 @@
       </c>
       <c r="Q5" t="inlineStr">
         <is>
-          <t>-10000,00</t>
+          <t>-10000.00</t>
         </is>
       </c>
       <c r="R5" t="inlineStr">
@@ -2300,8 +2304,10 @@
           <t>1224</t>
         </is>
       </c>
-      <c r="C6" s="2" t="n">
-        <v>43875</v>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>14/02/2020</t>
+        </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
@@ -2358,7 +2364,7 @@
       </c>
       <c r="O6" t="inlineStr">
         <is>
-          <t>0,00</t>
+          <t>0.00</t>
         </is>
       </c>
       <c r="P6" t="inlineStr">
@@ -2368,7 +2374,7 @@
       </c>
       <c r="Q6" t="inlineStr">
         <is>
-          <t>-10000,00</t>
+          <t>-10000.00</t>
         </is>
       </c>
       <c r="R6" t="inlineStr">
@@ -2388,8 +2394,10 @@
           <t>1225</t>
         </is>
       </c>
-      <c r="C7" s="2" t="n">
-        <v>43875</v>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>14/02/2020</t>
+        </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
@@ -2446,7 +2454,7 @@
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>0,00</t>
+          <t>0.00</t>
         </is>
       </c>
       <c r="P7" t="inlineStr">
@@ -2456,7 +2464,7 @@
       </c>
       <c r="Q7" t="inlineStr">
         <is>
-          <t>-10000,00</t>
+          <t>-10000.00</t>
         </is>
       </c>
       <c r="R7" t="inlineStr">
@@ -2476,8 +2484,10 @@
           <t>1250</t>
         </is>
       </c>
-      <c r="C8" s="2" t="n">
-        <v>43875</v>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>14/02/2020</t>
+        </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
@@ -2539,12 +2549,12 @@
       </c>
       <c r="P8" t="inlineStr">
         <is>
-          <t>0,00</t>
+          <t>0.00</t>
         </is>
       </c>
       <c r="Q8" t="inlineStr">
         <is>
-          <t>10000,00</t>
+          <t>10000.00</t>
         </is>
       </c>
       <c r="R8" t="inlineStr">
@@ -2564,8 +2574,10 @@
           <t>1251</t>
         </is>
       </c>
-      <c r="C9" s="2" t="n">
-        <v>43875</v>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>14/02/2020</t>
+        </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
@@ -2627,12 +2639,12 @@
       </c>
       <c r="P9" t="inlineStr">
         <is>
-          <t>0,00</t>
+          <t>0.00</t>
         </is>
       </c>
       <c r="Q9" t="inlineStr">
         <is>
-          <t>10000,00</t>
+          <t>10000.00</t>
         </is>
       </c>
       <c r="R9" t="inlineStr">
@@ -2652,8 +2664,10 @@
           <t>1276</t>
         </is>
       </c>
-      <c r="C10" s="2" t="n">
-        <v>43969</v>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>18/05/2020</t>
+        </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
@@ -2685,7 +2699,7 @@
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>52,4</t>
+          <t>52.4</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
@@ -2710,17 +2724,17 @@
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>0,00</t>
+          <t>0.00</t>
         </is>
       </c>
       <c r="P10" t="inlineStr">
         <is>
-          <t>52,4</t>
+          <t>52.4</t>
         </is>
       </c>
       <c r="Q10" t="inlineStr">
         <is>
-          <t>-52,40</t>
+          <t>-52.40</t>
         </is>
       </c>
       <c r="R10" t="inlineStr">
@@ -2740,8 +2754,10 @@
           <t>1279</t>
         </is>
       </c>
-      <c r="C11" s="2" t="n">
-        <v>43969</v>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>18/05/2020</t>
+        </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
@@ -2773,7 +2789,7 @@
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>52,4</t>
+          <t>52.4</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
@@ -2798,17 +2814,17 @@
       </c>
       <c r="O11" t="inlineStr">
         <is>
-          <t>0,00</t>
+          <t>0.00</t>
         </is>
       </c>
       <c r="P11" t="inlineStr">
         <is>
-          <t>52,4</t>
+          <t>52.4</t>
         </is>
       </c>
       <c r="Q11" t="inlineStr">
         <is>
-          <t>-52,40</t>
+          <t>-52.40</t>
         </is>
       </c>
       <c r="R11" t="inlineStr">
@@ -2828,8 +2844,10 @@
           <t>1276</t>
         </is>
       </c>
-      <c r="C12" s="2" t="n">
-        <v>43969</v>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>18/05/2020</t>
+        </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
@@ -2861,7 +2879,7 @@
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>52,4</t>
+          <t>52.4</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
@@ -2886,17 +2904,17 @@
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>52,4</t>
+          <t>52.4</t>
         </is>
       </c>
       <c r="P12" t="inlineStr">
         <is>
-          <t>0,00</t>
+          <t>0.00</t>
         </is>
       </c>
       <c r="Q12" t="inlineStr">
         <is>
-          <t>52,40</t>
+          <t>52.40</t>
         </is>
       </c>
       <c r="R12" t="inlineStr">
@@ -2916,8 +2934,10 @@
           <t>1279</t>
         </is>
       </c>
-      <c r="C13" s="2" t="n">
-        <v>43969</v>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>18/05/2020</t>
+        </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
@@ -2949,7 +2969,7 @@
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>52,4</t>
+          <t>52.4</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
@@ -2974,17 +2994,17 @@
       </c>
       <c r="O13" t="inlineStr">
         <is>
-          <t>52,4</t>
+          <t>52.4</t>
         </is>
       </c>
       <c r="P13" t="inlineStr">
         <is>
-          <t>0,00</t>
+          <t>0.00</t>
         </is>
       </c>
       <c r="Q13" t="inlineStr">
         <is>
-          <t>52,40</t>
+          <t>52.40</t>
         </is>
       </c>
       <c r="R13" t="inlineStr">
@@ -3004,8 +3024,10 @@
           <t>1621</t>
         </is>
       </c>
-      <c r="C14" s="2" t="n">
-        <v>43972</v>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>21/05/2020</t>
+        </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
@@ -3037,7 +3059,7 @@
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>232,5</t>
+          <t>232.5</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
@@ -3058,17 +3080,17 @@
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t>0,00</t>
+          <t>0.00</t>
         </is>
       </c>
       <c r="P14" t="inlineStr">
         <is>
-          <t>232,5</t>
+          <t>232.5</t>
         </is>
       </c>
       <c r="Q14" t="inlineStr">
         <is>
-          <t>-232,50</t>
+          <t>-232.50</t>
         </is>
       </c>
       <c r="R14" t="inlineStr">
@@ -3088,8 +3110,10 @@
           <t>1622</t>
         </is>
       </c>
-      <c r="C15" s="2" t="n">
-        <v>43972</v>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>21/05/2020</t>
+        </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
@@ -3121,7 +3145,7 @@
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>232,5</t>
+          <t>232.5</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
@@ -3142,17 +3166,17 @@
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>0,00</t>
+          <t>0.00</t>
         </is>
       </c>
       <c r="P15" t="inlineStr">
         <is>
-          <t>232,5</t>
+          <t>232.5</t>
         </is>
       </c>
       <c r="Q15" t="inlineStr">
         <is>
-          <t>-232,50</t>
+          <t>-232.50</t>
         </is>
       </c>
       <c r="R15" t="inlineStr">
@@ -3172,8 +3196,10 @@
           <t>1621</t>
         </is>
       </c>
-      <c r="C16" s="2" t="n">
-        <v>43972</v>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>21/05/2020</t>
+        </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
@@ -3205,7 +3231,7 @@
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>232,5</t>
+          <t>232.5</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
@@ -3226,17 +3252,17 @@
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>232,5</t>
+          <t>232.5</t>
         </is>
       </c>
       <c r="P16" t="inlineStr">
         <is>
-          <t>0,00</t>
+          <t>0.00</t>
         </is>
       </c>
       <c r="Q16" t="inlineStr">
         <is>
-          <t>232,50</t>
+          <t>232.50</t>
         </is>
       </c>
       <c r="R16" t="inlineStr">
@@ -3256,8 +3282,10 @@
           <t>1622</t>
         </is>
       </c>
-      <c r="C17" s="2" t="n">
-        <v>43972</v>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>21/05/2020</t>
+        </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
@@ -3289,7 +3317,7 @@
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>232,5</t>
+          <t>232.5</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
@@ -3310,17 +3338,17 @@
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t>232,5</t>
+          <t>232.5</t>
         </is>
       </c>
       <c r="P17" t="inlineStr">
         <is>
-          <t>0,00</t>
+          <t>0.00</t>
         </is>
       </c>
       <c r="Q17" t="inlineStr">
         <is>
-          <t>232,50</t>
+          <t>232.50</t>
         </is>
       </c>
       <c r="R17" t="inlineStr">
@@ -3383,17 +3411,17 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>0,00</t>
+          <t>0.00</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>0,00</t>
+          <t>0.00</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>-26249921,36</t>
+          <t>-26249921.36</t>
         </is>
       </c>
     </row>
@@ -3410,17 +3438,17 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>0,00</t>
+          <t>0.00</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>0,00</t>
+          <t>0.00</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>-1612627,37</t>
+          <t>-1612627.37</t>
         </is>
       </c>
     </row>
@@ -3437,17 +3465,17 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>0,00</t>
+          <t>0.00</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>0,00</t>
+          <t>0.00</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>-525074,35</t>
+          <t>-525074.35</t>
         </is>
       </c>
     </row>
@@ -3464,17 +3492,17 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>0,00</t>
+          <t>0.00</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>0,00</t>
+          <t>0.00</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>-5003078,66</t>
+          <t>-5003078.66</t>
         </is>
       </c>
     </row>
@@ -3491,17 +3519,17 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>0,00</t>
+          <t>0.00</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>0,00</t>
+          <t>0.00</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>-168238,73</t>
+          <t>-168238.73</t>
         </is>
       </c>
     </row>
@@ -3518,17 +3546,17 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>0,00</t>
+          <t>0.00</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>0,00</t>
+          <t>0.00</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>-1100006,10</t>
+          <t>-1100006.10</t>
         </is>
       </c>
     </row>
@@ -3545,17 +3573,17 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>0,00</t>
+          <t>0.00</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>0,00</t>
+          <t>0.00</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>-122207,63</t>
+          <t>-122207.63</t>
         </is>
       </c>
     </row>
@@ -3572,17 +3600,17 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>0,00</t>
+          <t>0.00</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>0,00</t>
+          <t>0.00</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>-3500844,15</t>
+          <t>-3500844.15</t>
         </is>
       </c>
     </row>
@@ -3599,17 +3627,17 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>0,00</t>
+          <t>0.00</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>0,00</t>
+          <t>0.00</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>-1411270,51</t>
+          <t>-1411270.51</t>
         </is>
       </c>
     </row>
@@ -3626,17 +3654,17 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>0,00</t>
+          <t>0.00</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>0,00</t>
+          <t>0.00</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>-1689174,42</t>
+          <t>-1689174.42</t>
         </is>
       </c>
     </row>
@@ -3653,17 +3681,17 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>0,00</t>
+          <t>0.00</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>0,00</t>
+          <t>0.00</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>-307062,47</t>
+          <t>-307062.47</t>
         </is>
       </c>
     </row>
@@ -3680,17 +3708,17 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>0,00</t>
+          <t>0.00</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>0,00</t>
+          <t>0.00</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>-1000000,00</t>
+          <t>-1000000.00</t>
         </is>
       </c>
     </row>
@@ -3707,17 +3735,17 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>0,00</t>
+          <t>0.00</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>0,00</t>
+          <t>0.00</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>-316076,78</t>
+          <t>-316076.78</t>
         </is>
       </c>
     </row>
@@ -3734,17 +3762,17 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>0,00</t>
+          <t>0.00</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>0,00</t>
+          <t>0.00</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>-84794,43</t>
+          <t>-84794.43</t>
         </is>
       </c>
     </row>
@@ -3761,17 +3789,17 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>0,00</t>
+          <t>0.00</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>0,00</t>
+          <t>0.00</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>-361963,72</t>
+          <t>-361963.72</t>
         </is>
       </c>
     </row>
@@ -3788,17 +3816,17 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>0,00</t>
+          <t>0.00</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>0,00</t>
+          <t>0.00</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>-39081,71</t>
+          <t>-39081.71</t>
         </is>
       </c>
     </row>
@@ -3815,17 +3843,17 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>0,00</t>
+          <t>0.00</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>0,00</t>
+          <t>0.00</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>-23604,23</t>
+          <t>-23604.23</t>
         </is>
       </c>
     </row>
@@ -3842,17 +3870,17 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>0,00</t>
+          <t>0.00</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>0,00</t>
+          <t>0.00</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>-799067,84</t>
+          <t>-799067.84</t>
         </is>
       </c>
     </row>
@@ -3869,17 +3897,17 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>0,00</t>
+          <t>0.00</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>0,00</t>
+          <t>0.00</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>-21624,22</t>
+          <t>-21624.22</t>
         </is>
       </c>
     </row>
@@ -3896,17 +3924,17 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>0,00</t>
+          <t>0.00</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>0,00</t>
+          <t>0.00</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>-4070,67</t>
+          <t>-4070.67</t>
         </is>
       </c>
     </row>
@@ -3923,17 +3951,17 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>0,00</t>
+          <t>0.00</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>0,00</t>
+          <t>0.00</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>-62310,20</t>
+          <t>-62310.20</t>
         </is>
       </c>
     </row>
@@ -3950,17 +3978,17 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>0,00</t>
+          <t>0.00</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>0,00</t>
+          <t>0.00</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>-336512,15</t>
+          <t>-336512.15</t>
         </is>
       </c>
     </row>
@@ -3977,17 +4005,17 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>0,00</t>
+          <t>0.00</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>0,00</t>
+          <t>0.00</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>-2955,00</t>
+          <t>-2955.00</t>
         </is>
       </c>
     </row>
@@ -4004,17 +4032,17 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>0,00</t>
+          <t>0.00</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>0,00</t>
+          <t>0.00</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>-7349703,23</t>
+          <t>-7349703.23</t>
         </is>
       </c>
     </row>
@@ -4031,17 +4059,17 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>0,00</t>
+          <t>0.00</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>0,00</t>
+          <t>0.00</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>-13919480,54</t>
+          <t>-13919480.54</t>
         </is>
       </c>
     </row>
@@ -4058,17 +4086,17 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>0,00</t>
+          <t>0.00</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>0,00</t>
+          <t>0.00</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>-1474936,44</t>
+          <t>-1474936.44</t>
         </is>
       </c>
     </row>
@@ -4085,17 +4113,17 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>0,00</t>
+          <t>0.00</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>0,00</t>
+          <t>0.00</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>-708333,23</t>
+          <t>-708333.23</t>
         </is>
       </c>
     </row>
@@ -4112,17 +4140,17 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>0,00</t>
+          <t>0.00</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>0,00</t>
+          <t>0.00</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>-321405,23</t>
+          <t>-321405.23</t>
         </is>
       </c>
     </row>
@@ -4139,17 +4167,17 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>0,00</t>
+          <t>0.00</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>0,00</t>
+          <t>0.00</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>-291814,20</t>
+          <t>-291814.20</t>
         </is>
       </c>
     </row>
@@ -4166,17 +4194,17 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>0,00</t>
+          <t>0.00</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>0,00</t>
+          <t>0.00</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>-2874350,51</t>
+          <t>-2874350.51</t>
         </is>
       </c>
     </row>
@@ -4193,17 +4221,17 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>0,00</t>
+          <t>0.00</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>0,00</t>
+          <t>0.00</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>-1269570,43</t>
+          <t>-1269570.43</t>
         </is>
       </c>
     </row>
@@ -4220,17 +4248,17 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>0,00</t>
+          <t>0.00</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>0,00</t>
+          <t>0.00</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>-1604291,42</t>
+          <t>-1604291.42</t>
         </is>
       </c>
     </row>
@@ -4247,17 +4275,17 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>0,00</t>
+          <t>0.00</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>0,00</t>
+          <t>0.00</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>-461592,30</t>
+          <t>-461592.30</t>
         </is>
       </c>
     </row>
@@ -4274,17 +4302,17 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>0,00</t>
+          <t>0.00</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>0,00</t>
+          <t>0.00</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>-60997,31</t>
+          <t>-60997.31</t>
         </is>
       </c>
     </row>
@@ -4301,17 +4329,17 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>0,00</t>
+          <t>0.00</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>0,00</t>
+          <t>0.00</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>-306846,64</t>
+          <t>-306846.64</t>
         </is>
       </c>
     </row>
@@ -4328,17 +4356,17 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>0,00</t>
+          <t>0.00</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>0,00</t>
+          <t>0.00</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>-155040,19</t>
+          <t>-155040.19</t>
         </is>
       </c>
     </row>
@@ -4355,17 +4383,17 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>0,00</t>
+          <t>0.00</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>0,00</t>
+          <t>0.00</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>-3461305,00</t>
+          <t>-3461305.00</t>
         </is>
       </c>
     </row>
@@ -4382,17 +4410,17 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>0,00</t>
+          <t>0.00</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>0,00</t>
+          <t>0.00</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>-19408,12</t>
+          <t>-19408.12</t>
         </is>
       </c>
     </row>
@@ -4409,17 +4437,17 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>0,00</t>
+          <t>0.00</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>0,00</t>
+          <t>0.00</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>-87240,94</t>
+          <t>-87240.94</t>
         </is>
       </c>
     </row>
@@ -4436,17 +4464,17 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>0,00</t>
+          <t>0.00</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>0,00</t>
+          <t>0.00</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>-105710,53</t>
+          <t>-105710.53</t>
         </is>
       </c>
     </row>
@@ -4463,17 +4491,17 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>0,00</t>
+          <t>0.00</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>0,00</t>
+          <t>0.00</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>-34230,96</t>
+          <t>-34230.96</t>
         </is>
       </c>
     </row>
@@ -4490,17 +4518,17 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>0,00</t>
+          <t>0.00</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>0,00</t>
+          <t>0.00</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>-63914,64</t>
+          <t>-63914.64</t>
         </is>
       </c>
     </row>
@@ -4517,17 +4545,17 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>0,00</t>
+          <t>0.00</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>0,00</t>
+          <t>0.00</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>-876800,00</t>
+          <t>-876800.00</t>
         </is>
       </c>
     </row>

</xml_diff>